<commit_message>
Enrich BIO 304 Video Tracker with per-topic URLs
Added three columns to the Video Tracker sheet:
  P. Lecture Page         - the per-topic one-pager (or '(not yet built)')
  Q. Spaced Recall        - deep-link to that topic's cards
  R. Lab Workbook         - the printable workbook

All cells are hyperlinks. As Scrubs records each video and pastes the YouTube
URL into column L, the tracker becomes a single source of truth showing every
working surface tied to that topic.

_enrich_video_tracker.py committed so future regeneration is reproducible.
</commit_message>
<xml_diff>
--- a/BIO-304-Video-Tracker.xlsx
+++ b/BIO-304-Video-Tracker.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -126,8 +126,26 @@
       <sz val="10"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF1E3D4C"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF5C6970"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -168,6 +186,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFAFAF9"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E3D4C"/>
+        <bgColor rgb="FF1E3D4C"/>
       </patternFill>
     </fill>
   </fills>
@@ -235,7 +259,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -528,6 +552,11 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -815,7 +844,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="21.75" customHeight="1" s="50">
       <c r="A5" s="54" t="inlineStr">
         <is>
@@ -867,7 +895,6 @@
       </c>
       <c r="F6" s="58" t="n"/>
     </row>
-    <row r="7"/>
     <row r="8" ht="21.75" customHeight="1" s="50">
       <c r="A8" s="59" t="inlineStr">
         <is>
@@ -3779,7 +3806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:R47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="49" min="1" max="1"/>
@@ -3794,6 +3821,9 @@
     <col width="7" customWidth="1" style="49" min="10" max="11"/>
     <col width="36" customWidth="1" style="49" min="12" max="13"/>
     <col width="30" customWidth="1" style="49" min="14" max="14"/>
+    <col width="42" customWidth="1" style="50" min="16" max="16"/>
+    <col width="56" customWidth="1" style="50" min="17" max="17"/>
+    <col width="56" customWidth="1" style="50" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="50">
@@ -3813,11 +3843,10 @@
     <row r="3" ht="31.5" customHeight="1" s="50">
       <c r="A3" s="53" t="inlineStr">
         <is>
-          <t>Paste video URLs in column L, note URLs in column M. Column N has the OpenStax reference. Pre-work nights: Mon, Tue, Thu, Fri. Wednesday is recall + lab. Topic ID in column C is what the engine matches on.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>Paste video URLs in column L, note URLs in column M. Column N has the OpenStax reference. Columns P, Q, R hold the lecture page, spaced-recall deep-link, and lab workbook URLs respectively. Pre-work nights: Mon, Tue, Thu, Fri. Wednesday is recall + lab. Topic ID in column C is what the engine matches on.</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="30" customHeight="1" s="50">
       <c r="A5" s="78" t="inlineStr">
         <is>
@@ -3892,6 +3921,21 @@
       <c r="O5" s="78" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="P5" s="98" t="inlineStr">
+        <is>
+          <t>Lecture Page</t>
+        </is>
+      </c>
+      <c r="Q5" s="98" t="inlineStr">
+        <is>
+          <t>Spaced Recall (deep-link)</t>
+        </is>
+      </c>
+      <c r="R5" s="98" t="inlineStr">
+        <is>
+          <t>Lab Workbook</t>
         </is>
       </c>
     </row>
@@ -3955,6 +3999,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P6" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/levels-of-organization.html</t>
+        </is>
+      </c>
+      <c r="Q6" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-levels-of-organization</t>
+        </is>
+      </c>
+      <c r="R6" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day01_levels-of-organization.html</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="39.75" customHeight="1" s="50">
       <c r="A7" s="69" t="n">
@@ -4016,6 +4075,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P7" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/anatomical-position.html</t>
+        </is>
+      </c>
+      <c r="Q7" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-anatomical-terminology</t>
+        </is>
+      </c>
+      <c r="R7" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day01_anatomical-terminology-and-body-regions.html</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="39.75" customHeight="1" s="50">
       <c r="A8" s="69" t="n">
@@ -4077,6 +4151,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P8" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/homeostasis-feedback.html</t>
+        </is>
+      </c>
+      <c r="Q8" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-homeostasis</t>
+        </is>
+      </c>
+      <c r="R8" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day02_homeostasis-and-feedback-loops.html</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="39.75" customHeight="1" s="50">
       <c r="A9" s="91" t="n">
@@ -4138,6 +4227,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P9" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q9" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-cell-structure</t>
+        </is>
+      </c>
+      <c r="R9" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day03_cell-structure-and-organelles.html</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="39.75" customHeight="1" s="50">
       <c r="A10" s="76" t="n">
@@ -4199,6 +4303,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P10" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q10" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-membrane-transport</t>
+        </is>
+      </c>
+      <c r="R10" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day04_membrane-transport.html</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="39.75" customHeight="1" s="50">
       <c r="A11" s="79" t="n">
@@ -4260,6 +4379,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P11" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q11" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-epithelial-tissue</t>
+        </is>
+      </c>
+      <c r="R11" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day05_epithelial-tissue-classification.html</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="39.75" customHeight="1" s="50">
       <c r="A12" s="69" t="n">
@@ -4321,6 +4455,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P12" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q12" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-connective-tissue</t>
+        </is>
+      </c>
+      <c r="R12" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day06_connective-tissues.html</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="39.75" customHeight="1" s="50">
       <c r="A13" s="69" t="n">
@@ -4382,6 +4531,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P13" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q13" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-muscle-nervous-tissue</t>
+        </is>
+      </c>
+      <c r="R13" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day07_muscle-and-nervous-tissue-overview.html</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="39.75" customHeight="1" s="50">
       <c r="A14" s="91" t="n">
@@ -4443,6 +4607,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P14" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q14" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-skin-layers</t>
+        </is>
+      </c>
+      <c r="R14" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day07_skin-structure-and-layers.html</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="39.75" customHeight="1" s="50">
       <c r="A15" s="76" t="n">
@@ -4504,6 +4683,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P15" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q15" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-skin-functions</t>
+        </is>
+      </c>
+      <c r="R15" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day08_skin-functions-and-accessory-structures.html</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="39.75" customHeight="1" s="50">
       <c r="A16" s="79" t="n">
@@ -4565,6 +4759,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P16" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q16" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-bone-tissue</t>
+        </is>
+      </c>
+      <c r="R16" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day09_bone-tissue-and-bone-growth.html</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="39.75" customHeight="1" s="50">
       <c r="A17" s="69" t="n">
@@ -4626,6 +4835,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P17" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q17" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-axial-skeleton</t>
+        </is>
+      </c>
+      <c r="R17" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day10_axial-skeleton.html</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="39.75" customHeight="1" s="50">
       <c r="A18" s="69" t="n">
@@ -4687,6 +4911,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P18" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q18" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-appendicular-skeleton</t>
+        </is>
+      </c>
+      <c r="R18" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day11_appendicular-skeleton.html</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="39.75" customHeight="1" s="50">
       <c r="A19" s="69" t="n">
@@ -4748,6 +4987,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P19" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q19" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-joints-movements</t>
+        </is>
+      </c>
+      <c r="R19" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day12_joints-and-body-movements.html</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="39.75" customHeight="1" s="50">
       <c r="A20" s="91" t="n">
@@ -4809,6 +5063,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P20" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q20" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-skeletal-muscle-microanatomy</t>
+        </is>
+      </c>
+      <c r="R20" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day13_skeletal-muscle-microanatomy.html</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="39.75" customHeight="1" s="50">
       <c r="A21" s="76" t="n">
@@ -4870,6 +5139,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P21" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q21" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-motor-units</t>
+        </is>
+      </c>
+      <c r="R21" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day13_motor-units-and-muscle-mechanics.html</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="39.75" customHeight="1" s="50">
       <c r="A22" s="76" t="n">
@@ -4931,6 +5215,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P22" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q22" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-sliding-filament</t>
+        </is>
+      </c>
+      <c r="R22" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day14_sliding-filament-and-the-cross-bridge-cycle.html</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="39.75" customHeight="1" s="50">
       <c r="A23" s="79" t="n">
@@ -4992,6 +5291,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P23" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q23" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-neurons-rmp</t>
+        </is>
+      </c>
+      <c r="R23" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day15_neurons-and-resting-membrane-potential.html</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="39.75" customHeight="1" s="50">
       <c r="A24" s="69" t="n">
@@ -5053,6 +5367,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P24" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q24" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-action-potentials</t>
+        </is>
+      </c>
+      <c r="R24" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day16_action-potentials-and-synaptic-transmission.html</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="39.75" customHeight="1" s="50">
       <c r="A25" s="69" t="n">
@@ -5114,6 +5443,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P25" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q25" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-cns-organization</t>
+        </is>
+      </c>
+      <c r="R25" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day17_cns-organization-brain-and-spinal-cord.html</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="39.75" customHeight="1" s="50">
       <c r="A26" s="69" t="n">
@@ -5175,6 +5519,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P26" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q26" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-pns-autonomic</t>
+        </is>
+      </c>
+      <c r="R26" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day18_pns-and-autonomic-nervous-system.html</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="39.75" customHeight="1" s="50">
       <c r="A27" s="91" t="n">
@@ -5236,6 +5595,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P27" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q27" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-vision</t>
+        </is>
+      </c>
+      <c r="R27" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day19_vision.html</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="39.75" customHeight="1" s="50">
       <c r="A28" s="76" t="n">
@@ -5297,6 +5671,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P28" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q28" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-hearing-equilibrium</t>
+        </is>
+      </c>
+      <c r="R28" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day19_hearing-and-equilibrium.html</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="39.75" customHeight="1" s="50">
       <c r="A29" s="79" t="n">
@@ -5358,6 +5747,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P29" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q29" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-hormone-mechanisms</t>
+        </is>
+      </c>
+      <c r="R29" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day20_hormone-mechanisms.html</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="39.75" customHeight="1" s="50">
       <c r="A30" s="69" t="n">
@@ -5419,6 +5823,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P30" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q30" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-major-glands</t>
+        </is>
+      </c>
+      <c r="R30" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day20_major-endocrine-glands.html</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="39.75" customHeight="1" s="50">
       <c r="A31" s="91" t="n">
@@ -5480,6 +5899,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P31" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q31" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-blood-composition</t>
+        </is>
+      </c>
+      <c r="R31" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day21_blood-composition-and-hemopoiesis.html</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="39.75" customHeight="1" s="50">
       <c r="A32" s="76" t="n">
@@ -5541,6 +5975,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P32" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q32" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-hemostasis-blood-typing</t>
+        </is>
+      </c>
+      <c r="R32" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day21_hemostasis-and-blood-typing.html</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="39.75" customHeight="1" s="50">
       <c r="A33" s="79" t="n">
@@ -5602,6 +6051,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P33" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q33" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-heart-cardiac-cycle</t>
+        </is>
+      </c>
+      <c r="R33" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day22_heart-anatomy-and-the-cardiac-cycle.html</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="39.75" customHeight="1" s="50">
       <c r="A34" s="69" t="n">
@@ -5663,6 +6127,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P34" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q34" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-conduction-ecg</t>
+        </is>
+      </c>
+      <c r="R34" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day23_cardiac-conduction-system.html</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="39.75" customHeight="1" s="50">
       <c r="A35" s="69" t="n">
@@ -5724,6 +6203,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P35" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q35" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-vessels-hemodynamics</t>
+        </is>
+      </c>
+      <c r="R35" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day24_blood-vessels-and-hemodynamics.html</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="39.75" customHeight="1" s="50">
       <c r="A36" s="91" t="n">
@@ -5785,6 +6279,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P36" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q36" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-lymphatic-innate</t>
+        </is>
+      </c>
+      <c r="R36" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day25_lymphatic-system-and-innate-immunity.html</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="39.75" customHeight="1" s="50">
       <c r="A37" s="76" t="n">
@@ -5846,6 +6355,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P37" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q37" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-adaptive-immunity</t>
+        </is>
+      </c>
+      <c r="R37" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day26_adaptive-immunity.html</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="39.75" customHeight="1" s="50">
       <c r="A38" s="79" t="n">
@@ -5907,6 +6431,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P38" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q38" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-resp-anatomy-mechanics</t>
+        </is>
+      </c>
+      <c r="R38" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day27_respiratory-anatomy-and-mechanics.html</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="39.75" customHeight="1" s="50">
       <c r="A39" s="69" t="n">
@@ -5968,6 +6507,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P39" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q39" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-gas-exchange-transport</t>
+        </is>
+      </c>
+      <c r="R39" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day27_gas-exchange-and-transport.html</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="39.75" customHeight="1" s="50">
       <c r="A40" s="91" t="n">
@@ -6029,6 +6583,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P40" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q40" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-gi-anatomy-motility</t>
+        </is>
+      </c>
+      <c r="R40" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day28_gi-tract-anatomy-and-motility.html</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="39.75" customHeight="1" s="50">
       <c r="A41" s="76" t="n">
@@ -6090,6 +6659,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P41" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q41" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-digestion-absorption</t>
+        </is>
+      </c>
+      <c r="R41" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day28_digestion-and-absorption.html</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="39.75" customHeight="1" s="50">
       <c r="A42" s="79" t="n">
@@ -6151,6 +6735,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P42" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q42" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-kidney-filtration</t>
+        </is>
+      </c>
+      <c r="R42" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day29_kidney-anatomy-and-glomerular-filtration.html</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="39.75" customHeight="1" s="50">
       <c r="A43" s="69" t="n">
@@ -6212,6 +6811,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P43" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q43" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-tubular-function</t>
+        </is>
+      </c>
+      <c r="R43" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day30_tubular-function-and-urine-concentration.html</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="39.75" customHeight="1" s="50">
       <c r="A44" s="69" t="n">
@@ -6273,6 +6887,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P44" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q44" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-fluid-acid-base</t>
+        </is>
+      </c>
+      <c r="R44" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day31_fluid-electrolyte-and-acid-base-balance.html</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="39.75" customHeight="1" s="50">
       <c r="A45" s="91" t="n">
@@ -6334,6 +6963,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P45" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q45" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-male-reproductive</t>
+        </is>
+      </c>
+      <c r="R45" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day31_male-reproductive-system.html</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="39.75" customHeight="1" s="50">
       <c r="A46" s="76" t="n">
@@ -6395,6 +7039,21 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="P46" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q46" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-female-reproductive</t>
+        </is>
+      </c>
+      <c r="R46" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day32_female-reproductive-system.html</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="39.75" customHeight="1" s="50">
       <c r="A47" s="76" t="n">
@@ -6454,6 +7113,21 @@
       <c r="O47" s="76" t="inlineStr">
         <is>
           <t>Pending</t>
+        </is>
+      </c>
+      <c r="P47" s="100" t="inlineStr">
+        <is>
+          <t>(not yet built)</t>
+        </is>
+      </c>
+      <c r="Q47" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/bio304-spaced-recall-prototype.html#topic=t-pregnancy-development</t>
+        </is>
+      </c>
+      <c r="R47" s="99" t="inlineStr">
+        <is>
+          <t>https://drsrennie-stack.github.io/nonmajors/workbook_day32_pregnancy-a-p-basics.html</t>
         </is>
       </c>
     </row>
@@ -6469,6 +7143,95 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId87"/>
+  </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -6513,7 +7276,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="27.75" customHeight="1" s="50">
       <c r="A5" s="61" t="inlineStr">
         <is>

</xml_diff>